<commit_message>
style: TEST 输出改用 console.debug()
fix: 修正 原神 歌单中的 不再年轻的村庄(轻策夜间) 的 cover 不正确的问题
chore(songs): 调整歌单内容
chore(minecraft): 更新 Minecraft 列车车站建设情况
</commit_message>
<xml_diff>
--- a/minecraft/data/列车车站规划.xlsx
+++ b/minecraft/data/列车车站规划.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Duckhome\projects\MSVS\Source\Repos\yazicbs.github.io.online\minecraft\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Duckhome\projects\MSVS\Source\Repos\yazicbs.github.io\minecraft\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A87F1B6-1150-4144-A40F-61CE278110F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33109BC3-B402-47F3-BB2C-0AB10F589137}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="53">
   <si>
     <t>图例：</t>
   </si>
@@ -85,12 +85,6 @@
     <t>衫林铁道局</t>
   </si>
   <si>
-    <t>雪衫之界</t>
-  </si>
-  <si>
-    <t>-&gt; (在建)</t>
-  </si>
-  <si>
     <t>------------------</t>
   </si>
   <si>
@@ -148,9 +142,6 @@
     <t>樱林村</t>
   </si>
   <si>
-    <t>X 暂未开放</t>
-  </si>
-  <si>
     <t>圆沙池</t>
   </si>
   <si>
@@ -158,9 +149,6 @@
   </si>
   <si>
     <t>橡木岛</t>
-  </si>
-  <si>
-    <t>⌋</t>
   </si>
   <si>
     <t>花桥</t>
@@ -172,6 +160,43 @@
   </si>
   <si>
     <t>蜂谷</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>-&gt;</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="20"/>
+        <color theme="1"/>
+        <rFont val="NLXJT"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>-&gt;</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>海桥</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>⌋</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>雪衫林</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">-&gt; </t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>瞭望塔</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -179,7 +204,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -213,6 +238,13 @@
       <sz val="20"/>
       <color theme="1"/>
       <name val="NLXJT"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="宋体"/>
       <family val="3"/>
       <charset val="134"/>
     </font>
@@ -293,7 +325,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -364,6 +396,18 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -372,6 +416,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF33CCFF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -641,18 +690,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BB14"/>
+  <dimension ref="A1:AZ14"/>
   <sheetFormatPr defaultColWidth="18.21875" defaultRowHeight="28.2" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="16384" width="18.21875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:54" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:52" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:54" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:52" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
@@ -675,7 +724,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:54" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:52" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C6" s="2" t="s">
         <v>8</v>
       </c>
@@ -689,7 +738,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:54" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:52" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E7" s="3" t="s">
         <v>10</v>
       </c>
@@ -730,7 +779,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:54" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:52" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K8" s="4" t="s">
         <v>14</v>
       </c>
@@ -741,7 +790,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:54" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:52" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="M9" s="9" t="s">
         <v>17</v>
       </c>
@@ -770,113 +819,116 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:54" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:52" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="O10" s="5" t="s">
         <v>18</v>
       </c>
       <c r="P10" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="Q10" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="R10" s="17" t="s">
-        <v>9</v>
+      <c r="Q10" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="R10" s="26" t="s">
+        <v>50</v>
       </c>
       <c r="S10" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="T10" s="17" t="s">
-        <v>22</v>
+      <c r="T10" s="27" t="s">
+        <v>51</v>
       </c>
       <c r="U10" s="5" t="s">
         <v>20</v>
       </c>
+      <c r="V10" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="W10" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="X10" s="26" t="s">
+        <v>52</v>
+      </c>
     </row>
-    <row r="11" spans="1:54" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:52" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="O11" s="6" t="s">
         <v>18</v>
       </c>
       <c r="AC11" s="22" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="AD11" s="18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AE11" s="18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AF11" s="18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AG11" s="18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AH11" s="18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AI11" s="18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AJ11" s="18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AK11" s="18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AL11" s="18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AM11" s="18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AN11" s="18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AO11" s="18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AP11" s="18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AQ11" s="18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AR11" s="18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AS11" s="18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AT11" s="18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AU11" s="18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AV11" s="18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AW11" s="18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AX11" s="18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AY11" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="AZ11" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="BA11" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="BB11" s="11" t="s">
-        <v>24</v>
+        <v>21</v>
+      </c>
+      <c r="AZ11" s="11" t="s">
+        <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:54" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:52" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="O12" s="10" t="s">
         <v>17</v>
       </c>
@@ -884,69 +936,75 @@
         <v>9</v>
       </c>
       <c r="Q12" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="R12" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="S12" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="T12" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="U12" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="R12" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="S12" s="6" t="s">
+      <c r="V12" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="W12" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="T12" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="U12" s="6" t="s">
+      <c r="X12" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="Y12" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="V12" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="W12" s="6" t="s">
+      <c r="Z12" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="AA12" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="X12" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="Y12" s="6" t="s">
+      <c r="AB12" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="AC12" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="AD12" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="AE12" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="Z12" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="AA12" s="6" t="s">
+      <c r="AF12" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="AG12" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="AH12" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="AI12" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="AZ12" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="AB12" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="AC12" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="AD12" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="AE12" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="AF12" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="AG12" s="21" t="s">
-        <v>47</v>
-      </c>
-      <c r="BB12" s="12" t="s">
-        <v>32</v>
-      </c>
     </row>
-    <row r="13" spans="1:54" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:52" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="Y13" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="BB13" s="12" t="s">
-        <v>32</v>
+        <v>27</v>
+      </c>
+      <c r="AZ13" s="12" t="s">
+        <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:54" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:52" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="Y14" s="13" t="s">
         <v>17</v>
       </c>
@@ -954,88 +1012,82 @@
         <v>9</v>
       </c>
       <c r="AA14" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="AB14" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="AC14" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="AD14" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="AE14" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="AB14" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="AC14" s="8" t="s">
+      <c r="AF14" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="AG14" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="AD14" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="AE14" s="8" t="s">
+      <c r="AH14" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="AI14" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="AF14" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="AG14" s="8" t="s">
+      <c r="AJ14" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="AK14" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="AH14" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="AI14" s="8" t="s">
+      <c r="AL14" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="AM14" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="AJ14" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="AK14" s="8" t="s">
+      <c r="AN14" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="AO14" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="AL14" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="AM14" s="8" t="s">
+      <c r="AP14" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="AQ14" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="AN14" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="AO14" s="8" t="s">
+      <c r="AR14" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="AS14" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="AT14" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="AU14" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="AP14" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="AQ14" s="8" t="s">
+      <c r="AV14" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="AW14" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="AR14" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="AS14" s="23" t="s">
+      <c r="AX14" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="AY14" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="AZ14" s="25" t="s">
         <v>49</v>
-      </c>
-      <c r="AT14" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="AU14" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="AV14" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="AW14" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="AX14" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="AY14" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="AZ14" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="BA14" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="BB14" s="11" t="s">
-        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>